<commit_message>
updated metamodel and schema
</commit_message>
<xml_diff>
--- a/laderr-rules-0.3.1.xlsx
+++ b/laderr-rules-0.3.1.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28227"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28324"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\FavatoBarcelosPP\Dev\laderr\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56821C77-B164-4084-9477-67CFA8D5BF72}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB3AF65F-8434-424A-9CB2-A0D4F5480F54}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{89084A5C-62F7-4402-9527-9AFD86D07F17}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{89084A5C-62F7-4402-9527-9AFD86D07F17}"/>
   </bookViews>
   <sheets>
     <sheet name="LaDeRR Rules" sheetId="1" r:id="rId1"/>
@@ -716,7 +716,7 @@
     </row>
   </sheetData>
   <conditionalFormatting sqref="D2:D6">
-    <cfRule type="duplicateValues" dxfId="0" priority="2"/>
+    <cfRule type="duplicateValues" dxfId="0" priority="3"/>
   </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>